<commit_message>
Update Ke hoach to chuyen mon THCS, TKB, LBG va Phan phoi chuong trinh
</commit_message>
<xml_diff>
--- a/TKB toàn trường CHECK - lần 2.1.xlsx
+++ b/TKB toàn trường CHECK - lần 2.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UNIGO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_03326137967898BE6403AC965B3A0E7EEB05F533" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E50D985-1C2C-4E8B-83DE-D8196FD2E4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4284" yWindow="1104" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TKB_LOP_SC" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="182">
   <si>
     <t>Tiểu học và THCS UNIGO
 Năm học 2026 - 2027
@@ -474,10 +474,6 @@
     <t>Robotics - 3A1</t>
   </si>
   <si>
-    <t>Robotics - 1A1
-Tin - TT3</t>
-  </si>
-  <si>
     <t>Robotics - 3C1</t>
   </si>
   <si>
@@ -566,13 +562,20 @@
   </si>
   <si>
     <t>Trùng tiết / Nhiều lớp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robotics - 1A1
+</t>
+  </si>
+  <si>
+    <t>Tin - TT3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Times New Roman"/>
@@ -673,8 +676,14 @@
       <color rgb="FFC65911"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -729,6 +738,18 @@
         <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="34">
     <border>
@@ -1183,7 +1204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1288,9 +1309,6 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1304,29 +1322,18 @@
     <xf numFmtId="0" fontId="16" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1334,10 +1341,8 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1347,6 +1352,25 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1646,57 +1670,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="56" t="s">
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
-      <c r="O1" s="50"/>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="50"/>
-      <c r="R1" s="50"/>
-      <c r="S1" s="50"/>
-      <c r="T1" s="50"/>
-      <c r="U1" s="50"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
+      <c r="N1" s="54"/>
+      <c r="O1" s="54"/>
+      <c r="P1" s="54"/>
+      <c r="Q1" s="54"/>
+      <c r="R1" s="54"/>
+      <c r="S1" s="54"/>
+      <c r="T1" s="54"/>
+      <c r="U1" s="54"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A2" s="50"/>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
-      <c r="M2" s="50"/>
-      <c r="N2" s="50"/>
-      <c r="O2" s="50"/>
-      <c r="P2" s="50"/>
-      <c r="Q2" s="50"/>
-      <c r="R2" s="50"/>
-      <c r="S2" s="50"/>
-      <c r="T2" s="50"/>
-      <c r="U2" s="50"/>
+      <c r="A2" s="54"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="54"/>
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
+      <c r="Q2" s="54"/>
+      <c r="R2" s="54"/>
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="U2" s="54"/>
       <c r="V2" s="2"/>
       <c r="W2" s="2"/>
       <c r="X2" s="3"/>
@@ -1728,64 +1752,64 @@
       <c r="X3" s="2"/>
     </row>
     <row r="4" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="47"/>
-      <c r="E4" s="46" t="s">
+      <c r="D4" s="46"/>
+      <c r="E4" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="47"/>
-      <c r="G4" s="46" t="s">
+      <c r="F4" s="46"/>
+      <c r="G4" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="47"/>
-      <c r="I4" s="46" t="s">
+      <c r="H4" s="46"/>
+      <c r="I4" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="47"/>
-      <c r="K4" s="46" t="s">
+      <c r="J4" s="46"/>
+      <c r="K4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="47"/>
-      <c r="M4" s="46" t="s">
+      <c r="L4" s="46"/>
+      <c r="M4" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="47"/>
-      <c r="O4" s="46" t="s">
+      <c r="N4" s="46"/>
+      <c r="O4" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="46" t="s">
+      <c r="P4" s="46"/>
+      <c r="Q4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="R4" s="47"/>
-      <c r="S4" s="46" t="s">
+      <c r="R4" s="46"/>
+      <c r="S4" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="T4" s="47"/>
-      <c r="U4" s="63" t="s">
+      <c r="T4" s="46"/>
+      <c r="U4" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="V4" s="64"/>
-      <c r="W4" s="46" t="s">
+      <c r="V4" s="58"/>
+      <c r="W4" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="X4" s="47"/>
-      <c r="Y4" s="48" t="s">
+      <c r="X4" s="46"/>
+      <c r="Y4" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="Z4" s="47"/>
-      <c r="AA4" s="48" t="s">
+      <c r="Z4" s="46"/>
+      <c r="AA4" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="AB4" s="47"/>
+      <c r="AB4" s="46"/>
       <c r="AC4" s="33" t="s">
         <v>17</v>
       </c>
@@ -1808,8 +1832,8 @@
       <c r="AL4" s="34"/>
     </row>
     <row r="5" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="58"/>
-      <c r="B5" s="58"/>
+      <c r="A5" s="52"/>
+      <c r="B5" s="52"/>
       <c r="C5" s="27" t="s">
         <v>22</v>
       </c>
@@ -1920,7 +1944,7 @@
       </c>
     </row>
     <row r="6" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="60">
+      <c r="A6" s="55">
         <v>2</v>
       </c>
       <c r="B6" s="5">
@@ -2020,7 +2044,7 @@
       <c r="AL6" s="26"/>
     </row>
     <row r="7" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="52"/>
+      <c r="A7" s="49"/>
       <c r="B7" s="9">
         <v>2</v>
       </c>
@@ -2124,7 +2148,7 @@
       </c>
     </row>
     <row r="8" spans="1:38" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="52"/>
+      <c r="A8" s="49"/>
       <c r="B8" s="9">
         <v>3</v>
       </c>
@@ -2230,7 +2254,7 @@
       <c r="AL8" s="25"/>
     </row>
     <row r="9" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="52"/>
+      <c r="A9" s="49"/>
       <c r="B9" s="9">
         <v>4</v>
       </c>
@@ -2330,7 +2354,7 @@
       <c r="AL9" s="25"/>
     </row>
     <row r="10" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="58"/>
+      <c r="A10" s="52"/>
       <c r="B10" s="10">
         <v>5</v>
       </c>
@@ -2378,7 +2402,7 @@
       <c r="AL10" s="26"/>
     </row>
     <row r="11" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="51">
+      <c r="A11" s="48">
         <v>3</v>
       </c>
       <c r="B11" s="5">
@@ -2480,7 +2504,7 @@
       <c r="AL11" s="26"/>
     </row>
     <row r="12" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="52"/>
+      <c r="A12" s="49"/>
       <c r="B12" s="9">
         <v>2</v>
       </c>
@@ -2584,7 +2608,7 @@
       <c r="AL12" s="25"/>
     </row>
     <row r="13" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="52"/>
+      <c r="A13" s="49"/>
       <c r="B13" s="9">
         <v>3</v>
       </c>
@@ -2687,7 +2711,7 @@
       <c r="AL13" s="25"/>
     </row>
     <row r="14" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="52"/>
+      <c r="A14" s="49"/>
       <c r="B14" s="9">
         <v>4</v>
       </c>
@@ -2789,7 +2813,7 @@
       </c>
     </row>
     <row r="15" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="53"/>
+      <c r="A15" s="50"/>
       <c r="B15" s="10">
         <v>5</v>
       </c>
@@ -2837,7 +2861,7 @@
       <c r="AL15" s="26"/>
     </row>
     <row r="16" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="51">
+      <c r="A16" s="48">
         <v>4</v>
       </c>
       <c r="B16" s="5">
@@ -2939,7 +2963,7 @@
       <c r="AL16" s="26"/>
     </row>
     <row r="17" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="52"/>
+      <c r="A17" s="49"/>
       <c r="B17" s="9">
         <v>2</v>
       </c>
@@ -3041,7 +3065,7 @@
       <c r="AL17" s="25"/>
     </row>
     <row r="18" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="52"/>
+      <c r="A18" s="49"/>
       <c r="B18" s="9">
         <v>3</v>
       </c>
@@ -3143,7 +3167,7 @@
       <c r="AL18" s="25"/>
     </row>
     <row r="19" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="52"/>
+      <c r="A19" s="49"/>
       <c r="B19" s="9">
         <v>4</v>
       </c>
@@ -3247,7 +3271,7 @@
       </c>
     </row>
     <row r="20" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="53"/>
+      <c r="A20" s="50"/>
       <c r="B20" s="10">
         <v>5</v>
       </c>
@@ -3295,7 +3319,7 @@
       <c r="AL20" s="26"/>
     </row>
     <row r="21" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="51">
+      <c r="A21" s="48">
         <v>5</v>
       </c>
       <c r="B21" s="5">
@@ -3380,7 +3404,7 @@
         <v>47</v>
       </c>
       <c r="AC21" s="25" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="AD21" s="25" t="s">
         <v>49</v>
@@ -3397,7 +3421,7 @@
       <c r="AL21" s="26"/>
     </row>
     <row r="22" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="52"/>
+      <c r="A22" s="49"/>
       <c r="B22" s="9">
         <v>2</v>
       </c>
@@ -3478,9 +3502,6 @@
       </c>
       <c r="AB22" s="25" t="s">
         <v>25</v>
-      </c>
-      <c r="AC22" s="25" t="s">
-        <v>76</v>
       </c>
       <c r="AD22" s="25" t="s">
         <v>25</v>
@@ -3501,7 +3522,7 @@
       <c r="AL22" s="25"/>
     </row>
     <row r="23" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="52"/>
+      <c r="A23" s="49"/>
       <c r="B23" s="9">
         <v>3</v>
       </c>
@@ -3603,7 +3624,7 @@
       <c r="AL23" s="25"/>
     </row>
     <row r="24" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="52"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="9">
         <v>4</v>
       </c>
@@ -3703,7 +3724,7 @@
       </c>
     </row>
     <row r="25" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="53"/>
+      <c r="A25" s="50"/>
       <c r="B25" s="10">
         <v>5</v>
       </c>
@@ -3751,7 +3772,7 @@
       <c r="AL25" s="26"/>
     </row>
     <row r="26" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="51">
+      <c r="A26" s="48">
         <v>6</v>
       </c>
       <c r="B26" s="5">
@@ -3853,7 +3874,7 @@
       <c r="AL26" s="26"/>
     </row>
     <row r="27" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="52"/>
+      <c r="A27" s="49"/>
       <c r="B27" s="9">
         <v>2</v>
       </c>
@@ -3959,7 +3980,7 @@
       </c>
     </row>
     <row r="28" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="52"/>
+      <c r="A28" s="49"/>
       <c r="B28" s="9">
         <v>3</v>
       </c>
@@ -4063,7 +4084,7 @@
       <c r="AL28" s="25"/>
     </row>
     <row r="29" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="52"/>
+      <c r="A29" s="49"/>
       <c r="B29" s="9">
         <v>4</v>
       </c>
@@ -4163,7 +4184,7 @@
       </c>
     </row>
     <row r="30" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="53"/>
+      <c r="A30" s="50"/>
       <c r="B30" s="10">
         <v>5</v>
       </c>
@@ -4211,7 +4232,7 @@
       <c r="AL30" s="26"/>
     </row>
     <row r="31" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="51">
+      <c r="A31" s="48">
         <v>7</v>
       </c>
       <c r="B31" s="5">
@@ -4243,7 +4264,7 @@
       <c r="Z31" s="20"/>
     </row>
     <row r="32" spans="1:38" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="52"/>
+      <c r="A32" s="49"/>
       <c r="B32" s="9">
         <v>2</v>
       </c>
@@ -4273,7 +4294,7 @@
       <c r="Z32" s="19"/>
     </row>
     <row r="33" spans="1:26" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="52"/>
+      <c r="A33" s="49"/>
       <c r="B33" s="9">
         <v>3</v>
       </c>
@@ -4303,7 +4324,7 @@
       <c r="Z33" s="19"/>
     </row>
     <row r="34" spans="1:26" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="52"/>
+      <c r="A34" s="49"/>
       <c r="B34" s="9">
         <v>4</v>
       </c>
@@ -4333,7 +4354,7 @@
       <c r="Z34" s="19"/>
     </row>
     <row r="35" spans="1:26" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="53"/>
+      <c r="A35" s="50"/>
       <c r="B35" s="10">
         <v>5</v>
       </c>
@@ -4363,16 +4384,16 @@
       <c r="Z35" s="21"/>
     </row>
     <row r="38" spans="1:26" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="61" t="s">
+      <c r="A38" s="62" t="s">
         <v>137</v>
       </c>
-      <c r="B38" s="50"/>
-      <c r="C38" s="50"/>
-      <c r="D38" s="50"/>
-      <c r="E38" s="50"/>
-      <c r="F38" s="50"/>
-      <c r="G38" s="50"/>
-      <c r="H38" s="50"/>
+      <c r="B38" s="54"/>
+      <c r="C38" s="54"/>
+      <c r="D38" s="54"/>
+      <c r="E38" s="54"/>
+      <c r="F38" s="54"/>
+      <c r="G38" s="54"/>
+      <c r="H38" s="54"/>
       <c r="I38" s="36"/>
       <c r="J38" s="36"/>
       <c r="K38" s="36"/>
@@ -4381,16 +4402,16 @@
       <c r="N38" s="36"/>
     </row>
     <row r="39" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="49" t="s">
+      <c r="A39" s="63" t="s">
         <v>138</v>
       </c>
-      <c r="B39" s="50"/>
-      <c r="C39" s="50"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="50"/>
-      <c r="F39" s="50"/>
-      <c r="G39" s="50"/>
-      <c r="H39" s="50"/>
+      <c r="B39" s="54"/>
+      <c r="C39" s="54"/>
+      <c r="D39" s="54"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="54"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="54"/>
       <c r="I39" s="36"/>
       <c r="J39" s="36"/>
       <c r="K39" s="36"/>
@@ -4447,7 +4468,7 @@
       <c r="N41" s="36"/>
     </row>
     <row r="42" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="54" t="s">
+      <c r="A42" s="59" t="s">
         <v>146</v>
       </c>
       <c r="B42" s="37" t="s">
@@ -4456,7 +4477,9 @@
       <c r="C42" s="38"/>
       <c r="D42" s="38"/>
       <c r="E42" s="38"/>
-      <c r="F42" s="38"/>
+      <c r="F42" s="65" t="s">
+        <v>181</v>
+      </c>
       <c r="G42" s="38"/>
       <c r="H42" s="38"/>
       <c r="I42" s="36"/>
@@ -4466,8 +4489,8 @@
       <c r="M42" s="36"/>
       <c r="N42" s="36"/>
     </row>
-    <row r="43" spans="1:26" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="55"/>
+    <row r="43" spans="1:26" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="60"/>
       <c r="B43" s="37" t="s">
         <v>148</v>
       </c>
@@ -4476,11 +4499,11 @@
       <c r="E43" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="F43" s="40" t="s">
+      <c r="F43" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="G43" s="39" t="s">
         <v>150</v>
-      </c>
-      <c r="G43" s="39" t="s">
-        <v>151</v>
       </c>
       <c r="H43" s="38"/>
       <c r="I43" s="36"/>
@@ -4491,20 +4514,20 @@
       <c r="N43" s="36"/>
     </row>
     <row r="44" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="55"/>
+      <c r="A44" s="60"/>
       <c r="B44" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="C44" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="C44" s="41" t="s">
+      <c r="D44" s="40" t="s">
         <v>153</v>
-      </c>
-      <c r="D44" s="41" t="s">
-        <v>154</v>
       </c>
       <c r="E44" s="38"/>
       <c r="F44" s="38"/>
-      <c r="G44" s="41" t="s">
-        <v>155</v>
+      <c r="G44" s="40" t="s">
+        <v>154</v>
       </c>
       <c r="H44" s="38"/>
       <c r="I44" s="36"/>
@@ -4515,24 +4538,24 @@
       <c r="N44" s="36"/>
     </row>
     <row r="45" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="55"/>
+      <c r="A45" s="60"/>
       <c r="B45" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="C45" s="40" t="s">
         <v>156</v>
       </c>
-      <c r="C45" s="41" t="s">
+      <c r="D45" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="D45" s="39" t="s">
+      <c r="E45" s="40" t="s">
         <v>158</v>
       </c>
-      <c r="E45" s="41" t="s">
+      <c r="F45" s="39" t="s">
         <v>159</v>
       </c>
-      <c r="F45" s="39" t="s">
+      <c r="G45" s="40" t="s">
         <v>160</v>
-      </c>
-      <c r="G45" s="41" t="s">
-        <v>161</v>
       </c>
       <c r="H45" s="38"/>
       <c r="I45" s="36"/>
@@ -4543,16 +4566,16 @@
       <c r="N45" s="36"/>
     </row>
     <row r="46" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="55"/>
+      <c r="A46" s="60"/>
       <c r="B46" s="37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C46" s="38"/>
       <c r="D46" s="38"/>
       <c r="E46" s="38"/>
       <c r="F46" s="38"/>
       <c r="G46" s="39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H46" s="38"/>
       <c r="I46" s="36"/>
@@ -4563,22 +4586,22 @@
       <c r="N46" s="36"/>
     </row>
     <row r="47" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="54" t="s">
-        <v>164</v>
+      <c r="A47" s="59" t="s">
+        <v>163</v>
       </c>
       <c r="B47" s="37" t="s">
         <v>147</v>
       </c>
       <c r="C47" s="38"/>
-      <c r="D47" s="41" t="s">
+      <c r="D47" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="E47" s="38"/>
+      <c r="F47" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="E47" s="38"/>
-      <c r="F47" s="41" t="s">
+      <c r="G47" s="40" t="s">
         <v>166</v>
-      </c>
-      <c r="G47" s="41" t="s">
-        <v>167</v>
       </c>
       <c r="H47" s="38"/>
       <c r="I47" s="36"/>
@@ -4589,20 +4612,20 @@
       <c r="N47" s="36"/>
     </row>
     <row r="48" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="55"/>
+      <c r="A48" s="60"/>
       <c r="B48" s="37" t="s">
         <v>148</v>
       </c>
       <c r="C48" s="38"/>
-      <c r="D48" s="41" t="s">
+      <c r="D48" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="E48" s="38"/>
+      <c r="F48" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="E48" s="38"/>
-      <c r="F48" s="41" t="s">
+      <c r="G48" s="39" t="s">
         <v>169</v>
-      </c>
-      <c r="G48" s="39" t="s">
-        <v>170</v>
       </c>
       <c r="H48" s="38"/>
       <c r="I48" s="36"/>
@@ -4613,22 +4636,22 @@
       <c r="N48" s="36"/>
     </row>
     <row r="49" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="55"/>
+      <c r="A49" s="60"/>
       <c r="B49" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="C49" s="38"/>
+      <c r="D49" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="C49" s="38"/>
-      <c r="D49" s="41" t="s">
-        <v>153</v>
-      </c>
-      <c r="E49" s="41" t="s">
+      <c r="E49" s="40" t="s">
+        <v>170</v>
+      </c>
+      <c r="F49" s="40" t="s">
         <v>171</v>
       </c>
-      <c r="F49" s="41" t="s">
+      <c r="G49" s="39" t="s">
         <v>172</v>
-      </c>
-      <c r="G49" s="39" t="s">
-        <v>173</v>
       </c>
       <c r="H49" s="38"/>
       <c r="I49" s="36"/>
@@ -4639,19 +4662,19 @@
       <c r="N49" s="36"/>
     </row>
     <row r="50" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="55"/>
+      <c r="A50" s="60"/>
       <c r="B50" s="37" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C50" s="38"/>
       <c r="D50" s="39" t="s">
+        <v>173</v>
+      </c>
+      <c r="E50" s="39" t="s">
         <v>174</v>
       </c>
-      <c r="E50" s="39" t="s">
+      <c r="F50" s="39" t="s">
         <v>175</v>
-      </c>
-      <c r="F50" s="39" t="s">
-        <v>176</v>
       </c>
       <c r="G50" s="38"/>
       <c r="H50" s="38"/>
@@ -4663,9 +4686,9 @@
       <c r="N50" s="36"/>
     </row>
     <row r="51" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="55"/>
+      <c r="A51" s="60"/>
       <c r="B51" s="37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C51" s="38"/>
       <c r="D51" s="38"/>
@@ -4697,8 +4720,8 @@
       <c r="N52" s="36"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="42" t="s">
-        <v>177</v>
+      <c r="A53" s="41" t="s">
+        <v>176</v>
       </c>
       <c r="B53" s="36"/>
       <c r="C53" s="36"/>
@@ -4715,16 +4738,16 @@
       <c r="N53" s="36"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="43" t="s">
+      <c r="A54" s="42" t="s">
+        <v>177</v>
+      </c>
+      <c r="B54" s="36"/>
+      <c r="C54" s="43" t="s">
         <v>178</v>
       </c>
-      <c r="B54" s="36"/>
-      <c r="C54" s="44" t="s">
+      <c r="D54" s="36"/>
+      <c r="E54" s="44" t="s">
         <v>179</v>
-      </c>
-      <c r="D54" s="36"/>
-      <c r="E54" s="45" t="s">
-        <v>180</v>
       </c>
       <c r="F54" s="36"/>
       <c r="G54" s="36"/>
@@ -4882,6 +4905,18 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="W4:X4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="A42:A46"/>
+    <mergeCell ref="A47:A51"/>
+    <mergeCell ref="A26:A30"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="F1:U1"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="Q4:R4"/>
     <mergeCell ref="A31:A35"/>
@@ -4898,18 +4933,6 @@
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="U4:V4"/>
-    <mergeCell ref="A47:A51"/>
-    <mergeCell ref="A26:A30"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="F1:U1"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="W4:X4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A21:A25"/>
-    <mergeCell ref="A42:A46"/>
   </mergeCells>
   <printOptions verticalCentered="1"/>
   <pageMargins left="0.4" right="0" top="0" bottom="0" header="0.5" footer="0.5"/>

</xml_diff>